<commit_message>
Update manuscript data, materials, figures and reproducible R analyses
</commit_message>
<xml_diff>
--- a/Exp_Material/Exp1/Pretest_Table.xlsx
+++ b/Exp_Material/Exp1/Pretest_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\lkz\bo\1\自己论文\论文1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A67FE75-5B82-479C-95E5-BF7A253036BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4A44F5-1AC6-4982-9C07-DDF7F8D980F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="59">
   <si>
     <t>认知需要量表（NFC）</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -258,6 +258,46 @@
   </si>
   <si>
     <t>信息性影响</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>主题涉入度（TI）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>拖延与我的日常生活密切相关</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>拖延这个问题对我来说很重要</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我经常思考拖延如何影响我的学习、工作或个人目标</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>理解拖延有助于改善我自己的行为</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>信息加工动机（MP）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我愿意认真思考与拖延有关的信息</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我有动力理解关于拖延文本中提出的原因和论点</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我愿意评估关于拖延的信息是否有说服力和有用</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我打算在阅读关于拖延的文本时保持注意</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -598,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="55.75" customWidth="1"/>
@@ -871,43 +911,109 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" ht="142.5" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="142.5" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B49" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="142.5" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>